<commit_message>
Calling snps for a sanity check
</commit_message>
<xml_diff>
--- a/genbank/SRA_metadata-taxonomy.xlsx
+++ b/genbank/SRA_metadata-taxonomy.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mac/github/lates-wgs/genbank/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A69524DF-968A-3249-A6AF-BB1AC1580BB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D898FE8-61A9-3442-B136-969BDF703794}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10000" yWindow="760" windowWidth="30240" windowHeight="17800" tabRatio="500" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-34400" yWindow="1740" windowWidth="30240" windowHeight="17800" tabRatio="500" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Contact Info and Instructions" sheetId="3" r:id="rId1"/>
@@ -230,7 +230,7 @@
           <rPr>
             <b/>
             <sz val="10"/>
-            <color indexed="81"/>
+            <color rgb="FF000000"/>
             <rFont val="Verdana"/>
             <family val="2"/>
           </rPr>
@@ -1601,36 +1601,6 @@
     <t>Fitzroy47-R1.fastq.gz</t>
   </si>
   <si>
-    <t>WAF004001 -R1.fastq.gz</t>
-  </si>
-  <si>
-    <t>WAF004002 -R1.fastq.gz</t>
-  </si>
-  <si>
-    <t>WAF004003 -R1.fastq.gz</t>
-  </si>
-  <si>
-    <t>WAF004008 -R1.fastq.gz</t>
-  </si>
-  <si>
-    <t>WAF004014 -R1.fastq.gz</t>
-  </si>
-  <si>
-    <t>WAF003767 -R1.fastq.gz</t>
-  </si>
-  <si>
-    <t>WAF003768 -R1.fastq.gz</t>
-  </si>
-  <si>
-    <t>WAF003770 -R1.fastq.gz</t>
-  </si>
-  <si>
-    <t>WAF003774 -R1.fastq.gz</t>
-  </si>
-  <si>
-    <t>WAF003775 -R1.fastq.gz</t>
-  </si>
-  <si>
     <t>Broome01-R2.fastq.gz</t>
   </si>
   <si>
@@ -1703,34 +1673,64 @@
     <t>Fitzroy47-R2.fastq.gz</t>
   </si>
   <si>
-    <t>WAF004001 -R2.fastq.gz</t>
-  </si>
-  <si>
-    <t>WAF004002 -R2.fastq.gz</t>
-  </si>
-  <si>
-    <t>WAF004003 -R2.fastq.gz</t>
-  </si>
-  <si>
-    <t>WAF004008 -R2.fastq.gz</t>
-  </si>
-  <si>
-    <t>WAF004014 -R2.fastq.gz</t>
-  </si>
-  <si>
-    <t>WAF003767 -R2.fastq.gz</t>
-  </si>
-  <si>
-    <t>WAF003768 -R2.fastq.gz</t>
-  </si>
-  <si>
-    <t>WAF003770 -R2.fastq.gz</t>
-  </si>
-  <si>
-    <t>WAF003774 -R2.fastq.gz</t>
-  </si>
-  <si>
-    <t>WAF003775 -R2.fastq.gz</t>
+    <t>WAF004001-R1.fastq.gz</t>
+  </si>
+  <si>
+    <t>WAF004002-R1.fastq.gz</t>
+  </si>
+  <si>
+    <t>WAF004003-R1.fastq.gz</t>
+  </si>
+  <si>
+    <t>WAF004008-R1.fastq.gz</t>
+  </si>
+  <si>
+    <t>WAF004014-R1.fastq.gz</t>
+  </si>
+  <si>
+    <t>WAF003767-R1.fastq.gz</t>
+  </si>
+  <si>
+    <t>WAF003768-R1.fastq.gz</t>
+  </si>
+  <si>
+    <t>WAF003770-R1.fastq.gz</t>
+  </si>
+  <si>
+    <t>WAF003774-R1.fastq.gz</t>
+  </si>
+  <si>
+    <t>WAF003775-R1.fastq.gz</t>
+  </si>
+  <si>
+    <t>WAF004001-R2.fastq.gz</t>
+  </si>
+  <si>
+    <t>WAF004002-R2.fastq.gz</t>
+  </si>
+  <si>
+    <t>WAF004003-R2.fastq.gz</t>
+  </si>
+  <si>
+    <t>WAF004008-R2.fastq.gz</t>
+  </si>
+  <si>
+    <t>WAF004014-R2.fastq.gz</t>
+  </si>
+  <si>
+    <t>WAF003767-R2.fastq.gz</t>
+  </si>
+  <si>
+    <t>WAF003768-R2.fastq.gz</t>
+  </si>
+  <si>
+    <t>WAF003770-R2.fastq.gz</t>
+  </si>
+  <si>
+    <t>WAF003774-R2.fastq.gz</t>
+  </si>
+  <si>
+    <t>WAF003775-R2.fastq.gz</t>
   </si>
 </sst>
 </file>
@@ -2205,6 +2205,9 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -2213,9 +2216,6 @@
     </xf>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="77">
@@ -3089,7 +3089,7 @@
         <v>362</v>
       </c>
       <c r="M2" s="13" t="s">
-        <v>396</v>
+        <v>386</v>
       </c>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.2">
@@ -3130,7 +3130,7 @@
         <v>363</v>
       </c>
       <c r="M3" s="13" t="s">
-        <v>397</v>
+        <v>387</v>
       </c>
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.2">
@@ -3171,7 +3171,7 @@
         <v>364</v>
       </c>
       <c r="M4" s="13" t="s">
-        <v>398</v>
+        <v>388</v>
       </c>
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.2">
@@ -3212,7 +3212,7 @@
         <v>365</v>
       </c>
       <c r="M5" s="13" t="s">
-        <v>399</v>
+        <v>389</v>
       </c>
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.2">
@@ -3253,7 +3253,7 @@
         <v>366</v>
       </c>
       <c r="M6" s="13" t="s">
-        <v>400</v>
+        <v>390</v>
       </c>
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.2">
@@ -3294,7 +3294,7 @@
         <v>367</v>
       </c>
       <c r="M7" s="13" t="s">
-        <v>401</v>
+        <v>391</v>
       </c>
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.2">
@@ -3335,7 +3335,7 @@
         <v>368</v>
       </c>
       <c r="M8" s="13" t="s">
-        <v>402</v>
+        <v>392</v>
       </c>
     </row>
     <row r="9" spans="1:17" x14ac:dyDescent="0.2">
@@ -3376,7 +3376,7 @@
         <v>369</v>
       </c>
       <c r="M9" s="13" t="s">
-        <v>403</v>
+        <v>393</v>
       </c>
     </row>
     <row r="10" spans="1:17" x14ac:dyDescent="0.2">
@@ -3417,7 +3417,7 @@
         <v>370</v>
       </c>
       <c r="M10" s="13" t="s">
-        <v>404</v>
+        <v>394</v>
       </c>
     </row>
     <row r="11" spans="1:17" x14ac:dyDescent="0.2">
@@ -3458,7 +3458,7 @@
         <v>371</v>
       </c>
       <c r="M11" s="13" t="s">
-        <v>405</v>
+        <v>395</v>
       </c>
     </row>
     <row r="12" spans="1:17" x14ac:dyDescent="0.2">
@@ -3499,7 +3499,7 @@
         <v>372</v>
       </c>
       <c r="M12" s="13" t="s">
-        <v>406</v>
+        <v>396</v>
       </c>
     </row>
     <row r="13" spans="1:17" x14ac:dyDescent="0.2">
@@ -3540,7 +3540,7 @@
         <v>373</v>
       </c>
       <c r="M13" s="13" t="s">
-        <v>407</v>
+        <v>397</v>
       </c>
     </row>
     <row r="14" spans="1:17" x14ac:dyDescent="0.2">
@@ -3581,7 +3581,7 @@
         <v>374</v>
       </c>
       <c r="M14" s="13" t="s">
-        <v>408</v>
+        <v>398</v>
       </c>
     </row>
     <row r="15" spans="1:17" x14ac:dyDescent="0.2">
@@ -3622,7 +3622,7 @@
         <v>375</v>
       </c>
       <c r="M15" s="13" t="s">
-        <v>409</v>
+        <v>399</v>
       </c>
     </row>
     <row r="16" spans="1:17" x14ac:dyDescent="0.2">
@@ -3663,7 +3663,7 @@
         <v>376</v>
       </c>
       <c r="M16" s="13" t="s">
-        <v>410</v>
+        <v>400</v>
       </c>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.2">
@@ -3704,7 +3704,7 @@
         <v>377</v>
       </c>
       <c r="M17" s="13" t="s">
-        <v>411</v>
+        <v>401</v>
       </c>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.2">
@@ -3745,7 +3745,7 @@
         <v>378</v>
       </c>
       <c r="M18" s="13" t="s">
-        <v>412</v>
+        <v>402</v>
       </c>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.2">
@@ -3786,7 +3786,7 @@
         <v>379</v>
       </c>
       <c r="M19" s="13" t="s">
-        <v>413</v>
+        <v>403</v>
       </c>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.2">
@@ -3827,7 +3827,7 @@
         <v>380</v>
       </c>
       <c r="M20" s="13" t="s">
-        <v>414</v>
+        <v>404</v>
       </c>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.2">
@@ -3868,7 +3868,7 @@
         <v>381</v>
       </c>
       <c r="M21" s="13" t="s">
-        <v>415</v>
+        <v>405</v>
       </c>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.2">
@@ -3909,7 +3909,7 @@
         <v>382</v>
       </c>
       <c r="M22" s="13" t="s">
-        <v>416</v>
+        <v>406</v>
       </c>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.2">
@@ -3950,7 +3950,7 @@
         <v>383</v>
       </c>
       <c r="M23" s="13" t="s">
-        <v>417</v>
+        <v>407</v>
       </c>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.2">
@@ -3991,7 +3991,7 @@
         <v>384</v>
       </c>
       <c r="M24" s="13" t="s">
-        <v>418</v>
+        <v>408</v>
       </c>
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.2">
@@ -4032,7 +4032,7 @@
         <v>385</v>
       </c>
       <c r="M25" s="13" t="s">
-        <v>419</v>
+        <v>409</v>
       </c>
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.2">
@@ -4070,7 +4070,7 @@
         <v>297</v>
       </c>
       <c r="L26" s="12" t="s">
-        <v>386</v>
+        <v>410</v>
       </c>
       <c r="M26" s="13" t="s">
         <v>420</v>
@@ -4111,7 +4111,7 @@
         <v>297</v>
       </c>
       <c r="L27" s="12" t="s">
-        <v>387</v>
+        <v>411</v>
       </c>
       <c r="M27" s="13" t="s">
         <v>421</v>
@@ -4152,7 +4152,7 @@
         <v>297</v>
       </c>
       <c r="L28" s="12" t="s">
-        <v>388</v>
+        <v>412</v>
       </c>
       <c r="M28" s="13" t="s">
         <v>422</v>
@@ -4193,7 +4193,7 @@
         <v>297</v>
       </c>
       <c r="L29" s="12" t="s">
-        <v>389</v>
+        <v>413</v>
       </c>
       <c r="M29" s="13" t="s">
         <v>423</v>
@@ -4234,7 +4234,7 @@
         <v>297</v>
       </c>
       <c r="L30" s="12" t="s">
-        <v>390</v>
+        <v>414</v>
       </c>
       <c r="M30" s="13" t="s">
         <v>424</v>
@@ -4275,7 +4275,7 @@
         <v>297</v>
       </c>
       <c r="L31" s="12" t="s">
-        <v>391</v>
+        <v>415</v>
       </c>
       <c r="M31" s="13" t="s">
         <v>425</v>
@@ -4316,7 +4316,7 @@
         <v>297</v>
       </c>
       <c r="L32" s="12" t="s">
-        <v>392</v>
+        <v>416</v>
       </c>
       <c r="M32" s="13" t="s">
         <v>426</v>
@@ -4357,7 +4357,7 @@
         <v>297</v>
       </c>
       <c r="L33" s="12" t="s">
-        <v>393</v>
+        <v>417</v>
       </c>
       <c r="M33" s="13" t="s">
         <v>427</v>
@@ -4398,7 +4398,7 @@
         <v>297</v>
       </c>
       <c r="L34" s="12" t="s">
-        <v>394</v>
+        <v>418</v>
       </c>
       <c r="M34" s="13" t="s">
         <v>428</v>
@@ -4439,7 +4439,7 @@
         <v>297</v>
       </c>
       <c r="L35" s="12" t="s">
-        <v>395</v>
+        <v>419</v>
       </c>
       <c r="M35" s="13" t="s">
         <v>429</v>
@@ -6778,8 +6778,8 @@
       <c r="A2" s="16" t="s">
         <v>37</v>
       </c>
-      <c r="B2" s="42"/>
-      <c r="C2" s="43"/>
+      <c r="B2" s="43"/>
+      <c r="C2" s="44"/>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
       <c r="F2" s="1"/>
@@ -7093,10 +7093,10 @@
       <c r="A37" s="2" t="s">
         <v>283</v>
       </c>
-      <c r="B37" s="44" t="s">
+      <c r="B37" s="45" t="s">
         <v>284</v>
       </c>
-      <c r="C37" s="44"/>
+      <c r="C37" s="45"/>
       <c r="D37" s="34"/>
       <c r="E37" s="34"/>
       <c r="F37" s="34"/>
@@ -7141,11 +7141,11 @@
       <c r="A42" s="2" t="s">
         <v>289</v>
       </c>
-      <c r="B42" s="44" t="s">
+      <c r="B42" s="45" t="s">
         <v>290</v>
       </c>
-      <c r="C42" s="44"/>
-      <c r="D42" s="44"/>
+      <c r="C42" s="45"/>
+      <c r="D42" s="45"/>
       <c r="E42" s="34"/>
       <c r="F42" s="34"/>
       <c r="G42" s="34"/>
@@ -7169,8 +7169,8 @@
       <c r="A45" s="16" t="s">
         <v>38</v>
       </c>
-      <c r="B45" s="42"/>
-      <c r="C45" s="43"/>
+      <c r="B45" s="43"/>
+      <c r="C45" s="44"/>
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A46" s="28" t="s">
@@ -7253,7 +7253,7 @@
       <c r="A56" s="16" t="s">
         <v>39</v>
       </c>
-      <c r="B56" s="45"/>
+      <c r="B56" s="42"/>
       <c r="C56" s="41"/>
     </row>
     <row r="57" spans="1:3" ht="25.5" customHeight="1" x14ac:dyDescent="0.15">
@@ -7956,40 +7956,25 @@
     <sortCondition ref="J93"/>
   </sortState>
   <mergeCells count="65">
-    <mergeCell ref="B68:C68"/>
-    <mergeCell ref="B69:C69"/>
-    <mergeCell ref="B70:C70"/>
-    <mergeCell ref="B62:C62"/>
-    <mergeCell ref="B63:C63"/>
-    <mergeCell ref="B64:C64"/>
-    <mergeCell ref="B65:C65"/>
-    <mergeCell ref="B66:C66"/>
-    <mergeCell ref="B67:C67"/>
-    <mergeCell ref="B61:C61"/>
-    <mergeCell ref="B50:C50"/>
-    <mergeCell ref="B51:C51"/>
-    <mergeCell ref="B54:C54"/>
-    <mergeCell ref="B55:C55"/>
-    <mergeCell ref="B56:C56"/>
-    <mergeCell ref="B57:C57"/>
-    <mergeCell ref="B58:C58"/>
-    <mergeCell ref="B59:C59"/>
-    <mergeCell ref="B60:C60"/>
-    <mergeCell ref="B24:C24"/>
-    <mergeCell ref="B49:C49"/>
-    <mergeCell ref="B43:C43"/>
-    <mergeCell ref="B44:C44"/>
-    <mergeCell ref="B45:C45"/>
-    <mergeCell ref="B46:C46"/>
-    <mergeCell ref="B47:C47"/>
-    <mergeCell ref="B48:C48"/>
-    <mergeCell ref="B37:C37"/>
-    <mergeCell ref="B42:D42"/>
-    <mergeCell ref="B19:C19"/>
-    <mergeCell ref="B20:C20"/>
-    <mergeCell ref="B21:C21"/>
-    <mergeCell ref="B22:C22"/>
-    <mergeCell ref="B23:C23"/>
+    <mergeCell ref="B81:C81"/>
+    <mergeCell ref="B82:C82"/>
+    <mergeCell ref="B83:C83"/>
+    <mergeCell ref="B76:C76"/>
+    <mergeCell ref="B77:C77"/>
+    <mergeCell ref="B78:C78"/>
+    <mergeCell ref="B79:C79"/>
+    <mergeCell ref="B80:C80"/>
+    <mergeCell ref="B71:C71"/>
+    <mergeCell ref="B72:C72"/>
+    <mergeCell ref="B73:C73"/>
+    <mergeCell ref="B74:C74"/>
+    <mergeCell ref="B75:C75"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="B1:C1"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="B5:C5"/>
     <mergeCell ref="B18:C18"/>
     <mergeCell ref="B7:C7"/>
     <mergeCell ref="B8:C8"/>
@@ -8002,25 +7987,40 @@
     <mergeCell ref="B15:C15"/>
     <mergeCell ref="B16:C16"/>
     <mergeCell ref="B17:C17"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="B1:C1"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="B3:C3"/>
-    <mergeCell ref="B4:C4"/>
-    <mergeCell ref="B5:C5"/>
-    <mergeCell ref="B71:C71"/>
-    <mergeCell ref="B72:C72"/>
-    <mergeCell ref="B73:C73"/>
-    <mergeCell ref="B74:C74"/>
-    <mergeCell ref="B75:C75"/>
-    <mergeCell ref="B81:C81"/>
-    <mergeCell ref="B82:C82"/>
-    <mergeCell ref="B83:C83"/>
-    <mergeCell ref="B76:C76"/>
-    <mergeCell ref="B77:C77"/>
-    <mergeCell ref="B78:C78"/>
-    <mergeCell ref="B79:C79"/>
-    <mergeCell ref="B80:C80"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="B21:C21"/>
+    <mergeCell ref="B22:C22"/>
+    <mergeCell ref="B23:C23"/>
+    <mergeCell ref="B24:C24"/>
+    <mergeCell ref="B49:C49"/>
+    <mergeCell ref="B43:C43"/>
+    <mergeCell ref="B44:C44"/>
+    <mergeCell ref="B45:C45"/>
+    <mergeCell ref="B46:C46"/>
+    <mergeCell ref="B47:C47"/>
+    <mergeCell ref="B48:C48"/>
+    <mergeCell ref="B37:C37"/>
+    <mergeCell ref="B42:D42"/>
+    <mergeCell ref="B61:C61"/>
+    <mergeCell ref="B50:C50"/>
+    <mergeCell ref="B51:C51"/>
+    <mergeCell ref="B54:C54"/>
+    <mergeCell ref="B55:C55"/>
+    <mergeCell ref="B56:C56"/>
+    <mergeCell ref="B57:C57"/>
+    <mergeCell ref="B58:C58"/>
+    <mergeCell ref="B59:C59"/>
+    <mergeCell ref="B60:C60"/>
+    <mergeCell ref="B68:C68"/>
+    <mergeCell ref="B69:C69"/>
+    <mergeCell ref="B70:C70"/>
+    <mergeCell ref="B62:C62"/>
+    <mergeCell ref="B63:C63"/>
+    <mergeCell ref="B64:C64"/>
+    <mergeCell ref="B65:C65"/>
+    <mergeCell ref="B66:C66"/>
+    <mergeCell ref="B67:C67"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>